<commit_message>
Change line 76 of example 8-4-1 to be nonlinear
</commit_message>
<xml_diff>
--- a/Lectures/Ex6-3-integer.xlsx
+++ b/Lectures/Ex6-3-integer.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\Box\_Rosenberg2024\Classes\CEE6410\Fall2024\CEE6410-Rosenberg-GitHub\CEE-6410-Rosenberg\Lectures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8B6E8260-3A9E-455D-BC83-F8D4F55E5295}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{86E4E2DF-3983-4A57-AF89-AA995C67B3E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="380" windowWidth="14400" windowHeight="7270" xr2:uid="{35A42BA3-A083-43AE-85BB-24EE6E7B125F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{77DE618E-983A-44DA-9869-006947BA4E0A}"/>
   </bookViews>
   <sheets>
     <sheet name="Table of Contents" sheetId="14" r:id="rId1"/>
@@ -29,7 +29,7 @@
     <sheet name="X" sheetId="1" r:id="rId14"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">CapCost!$A$3:$B$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">CapCost!$A$3:$B$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">I!$A$3:$E$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">IntLowBound!$A$3:$E$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">IntUpBnd!$A$3:$B$5</definedName>
@@ -58,12 +58,15 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="2"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="61">
   <si>
     <t>X</t>
   </si>
@@ -171,6 +174,9 @@
   </si>
   <si>
     <t>binary decision to build or do prject from source src (1=yes 0=no)</t>
+  </si>
+  <si>
+    <t>EPS</t>
   </si>
   <si>
     <t>CapCost</t>
@@ -625,50 +631,50 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D8782C3-A58E-4681-A837-9B5C47AA2B4A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36C4132D-7116-4AFC-837E-C68CA6CFFEB3}">
   <dimension ref="A1:E18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -677,7 +683,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -685,7 +691,7 @@
         <v>34</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -699,10 +705,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -711,7 +717,7 @@
         <v>0</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
@@ -719,7 +725,7 @@
         <v>32</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -736,7 +742,7 @@
         <v>30</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C7">
         <v>1</v>
@@ -753,7 +759,7 @@
         <v>28</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -770,7 +776,7 @@
         <v>26</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -787,7 +793,7 @@
         <v>24</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -801,10 +807,10 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -813,7 +819,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
@@ -821,7 +827,7 @@
         <v>22</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C12">
         <v>1</v>
@@ -838,7 +844,7 @@
         <v>20</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C13">
         <v>1</v>
@@ -855,7 +861,7 @@
         <v>17</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -872,7 +878,7 @@
         <v>3</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C15">
         <v>1</v>
@@ -886,10 +892,10 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -898,15 +904,15 @@
         <v>1</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C17">
         <v>0</v>
@@ -915,7 +921,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
@@ -923,7 +929,7 @@
         <v>0</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C18">
         <v>1</v>
@@ -937,29 +943,29 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" location="CapCost!A1" display="CapCost" xr:uid="{43DBE49E-DE99-406B-9A2B-2063735C0EAE}"/>
-    <hyperlink ref="A3" location="Scalar!A1" display="COST" xr:uid="{7EA3F94B-F3FF-4F62-92E0-851C13BA6C6E}"/>
-    <hyperlink ref="A4" location="I!A1" display="I" xr:uid="{24C9B348-4719-4348-B3CC-CB27E5DA09D1}"/>
-    <hyperlink ref="A6" location="IntLowBound!A1" display="IntLowBound" xr:uid="{084A2665-7C41-40AC-8E64-48B7BAC7F1A8}"/>
-    <hyperlink ref="A7" location="IntUpBnd!A1" display="IntUpBnd" xr:uid="{BD9232C3-D9BF-418B-A31E-6ABCEFDECC09}"/>
-    <hyperlink ref="A8" location="IntUpBound!A1" display="IntUpBound" xr:uid="{6A491867-67DF-40EE-86F2-0FEC24A73FAC}"/>
-    <hyperlink ref="A9" location="MaxCap!A1" display="MaxCap" xr:uid="{7C7E90FA-A541-4F84-AB7A-D8B59E6218EE}"/>
-    <hyperlink ref="A10" location="MaxCapacity!A1" display="MaxCapacity" xr:uid="{8EA52FD3-69D9-4E29-966F-A935F2D93E0C}"/>
-    <hyperlink ref="A11" location="Scalar!A1" display="MeetDemand" xr:uid="{C07D1735-CA0C-42A3-A288-2305073D5764}"/>
-    <hyperlink ref="A12" location="MinReqUse!A1" display="MinReqUse" xr:uid="{DF887249-268D-4968-9C80-7DA3F9FF75D7}"/>
-    <hyperlink ref="A13" location="MinUse!A1" display="MinUse" xr:uid="{9B837F35-4524-4976-8C58-072A85F00AFD}"/>
-    <hyperlink ref="A14" location="OpCost!A1" display="OpCost" xr:uid="{C7F4D79E-67FB-4456-BB50-EB660F35BBEB}"/>
-    <hyperlink ref="A15" location="src!A1" display="src" xr:uid="{F43BD174-0DAC-4D08-A01B-25C96964EF13}"/>
-    <hyperlink ref="A16" location="Scalar!A1" display="TCOST" xr:uid="{9F1D31FC-C779-4C4F-9A8B-6FEF943B9B53}"/>
-    <hyperlink ref="A17" location="Scalar!A1" display="TotDemand" xr:uid="{0591591C-1050-4A6E-9907-DBD6D82898EC}"/>
-    <hyperlink ref="A18" location="X!A1" display="X" xr:uid="{3FD847C5-AC47-4D36-8028-3BD28805DB3A}"/>
+    <hyperlink ref="A2" location="CapCost!A1" display="CapCost" xr:uid="{E2660445-CD8B-46C2-ABF6-EF37822B69F8}"/>
+    <hyperlink ref="A3" location="Scalar!A1" display="COST" xr:uid="{13D98F58-C89C-428E-AF5F-FC58BE66C544}"/>
+    <hyperlink ref="A4" location="I!A1" display="I" xr:uid="{B9C65DAA-1498-4029-A98C-0DEE0A5DE854}"/>
+    <hyperlink ref="A6" location="IntLowBound!A1" display="IntLowBound" xr:uid="{0895518D-9852-49F8-AB17-945DE7AAAFD9}"/>
+    <hyperlink ref="A7" location="IntUpBnd!A1" display="IntUpBnd" xr:uid="{A4E2CC11-E5ED-4A1E-B793-50BA0E5BC2E3}"/>
+    <hyperlink ref="A8" location="IntUpBound!A1" display="IntUpBound" xr:uid="{5869BCBC-7BF7-4781-944A-8E51D1C3B8B7}"/>
+    <hyperlink ref="A9" location="MaxCap!A1" display="MaxCap" xr:uid="{88FF868E-1863-42AA-84E8-AF116618C351}"/>
+    <hyperlink ref="A10" location="MaxCapacity!A1" display="MaxCapacity" xr:uid="{FDD79116-735F-4DF9-AB2F-64DBB30D4138}"/>
+    <hyperlink ref="A11" location="Scalar!A1" display="MeetDemand" xr:uid="{2DABF829-FCE3-4F1B-A0F7-E19984560350}"/>
+    <hyperlink ref="A12" location="MinReqUse!A1" display="MinReqUse" xr:uid="{E8F5BBA2-342E-4A9E-B00F-5C2B1D0F2353}"/>
+    <hyperlink ref="A13" location="MinUse!A1" display="MinUse" xr:uid="{65E9AD52-1DE2-49B8-AEFC-B922798BFE55}"/>
+    <hyperlink ref="A14" location="OpCost!A1" display="OpCost" xr:uid="{07B0CA8D-B6FB-450B-A429-5FFBEE4098BC}"/>
+    <hyperlink ref="A15" location="src!A1" display="src" xr:uid="{B1C9A889-F35E-4418-9A0B-D758FDAE5E8A}"/>
+    <hyperlink ref="A16" location="Scalar!A1" display="TCOST" xr:uid="{2D8EC73C-CCD9-449A-8157-804A2A1A8039}"/>
+    <hyperlink ref="A17" location="Scalar!A1" display="TotDemand" xr:uid="{E36EBFAA-34A4-486A-8755-5F0759076943}"/>
+    <hyperlink ref="A18" location="X!A1" display="X" xr:uid="{9573C3D0-DA7E-4F30-9589-503C7F73996A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD2FA05F-ED9B-4D04-A451-05214EEB3CA7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{092810AE-6520-4DD6-83B7-8A22C4422C9A}">
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1007,7 +1013,7 @@
         <v>0</v>
       </c>
       <c r="C4">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="D4" t="s">
         <v>9</v>
@@ -1024,7 +1030,7 @@
         <v>0</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="D5" t="s">
         <v>9</v>
@@ -1034,16 +1040,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:E5" xr:uid="{CD2FA05F-ED9B-4D04-A451-05214EEB3CA7}"/>
+  <autoFilter ref="A3:E5" xr:uid="{092810AE-6520-4DD6-83B7-8A22C4422C9A}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{C5F76D0F-E7C9-4D69-BC45-C9C4D2D5F3B5}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{86FBE176-6FB3-4EE1-8B6C-59BE3A598E9F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13A57599-D028-49E2-A3F6-6CA5FFD7C8DD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DD1AF31-BEB1-47C9-BF22-58B5C655B1BF}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1083,16 +1089,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:B4" xr:uid="{13A57599-D028-49E2-A3F6-6CA5FFD7C8DD}"/>
+  <autoFilter ref="A3:B4" xr:uid="{3DD1AF31-BEB1-47C9-BF22-58B5C655B1BF}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{3C230E39-A385-47F6-A12C-C2AEEAD65C6A}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{962B5F62-C43B-4A18-ABC4-F9474C4225F2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D1EC284-D29E-4E50-B901-486138948A5A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4761ADC-842A-4F73-92CF-58E9BBFFC553}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1140,16 +1146,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:B5" xr:uid="{8D1EC284-D29E-4E50-B901-486138948A5A}"/>
+  <autoFilter ref="A3:B5" xr:uid="{E4761ADC-842A-4F73-92CF-58E9BBFFC553}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{EFD111D4-D437-479E-9E53-50760D424FCA}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{7FC7666C-A197-4F96-AC3F-9456C15BAF79}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7090E77A-1C41-4C15-A231-C1BBC2E80E61}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B547B726-5999-476A-A2AC-089A6E2588B9}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1194,16 +1200,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:A5" xr:uid="{7090E77A-1C41-4C15-A231-C1BBC2E80E61}"/>
+  <autoFilter ref="A3:A5" xr:uid="{B547B726-5999-476A-A2AC-089A6E2588B9}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{DFF44EC1-A68C-49C3-8D1C-53152D84C21C}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{3305DCDB-F4ED-4235-BDD1-2934D77C300A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C99C21B1-49C9-4710-82B7-C4EAEA191ECF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{219D7CD9-24D6-4B13-B0FC-8E339F514A90}">
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1251,7 +1257,7 @@
         <v>0</v>
       </c>
       <c r="C4">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="D4" t="s">
         <v>9</v>
@@ -1268,26 +1274,26 @@
         <v>0</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="D5" t="s">
         <v>9</v>
       </c>
       <c r="E5">
-        <v>30</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:E5" xr:uid="{C99C21B1-49C9-4710-82B7-C4EAEA191ECF}"/>
+  <autoFilter ref="A3:E5" xr:uid="{219D7CD9-24D6-4B13-B0FC-8E339F514A90}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{51AB4C8B-5900-4D8C-A890-793DA39B6360}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{11EAC896-D99D-4853-AECA-916A83ED76EF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A71C7E0-2ADD-4EEA-89FD-813A077C81C7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5BEBEC9-BAF3-4C57-9F4B-0B61AF561DBB}">
   <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -1298,29 +1304,29 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B3">
         <v>2000</v>
       </c>
       <c r="C3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B5" t="s">
         <v>4</v>
@@ -1335,18 +1341,18 @@
         <v>7</v>
       </c>
       <c r="F5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B6" t="s">
         <v>27</v>
       </c>
       <c r="C6">
-        <v>330000</v>
+        <v>300000</v>
       </c>
       <c r="D6" t="s">
         <v>9</v>
@@ -1355,12 +1361,12 @@
         <v>0</v>
       </c>
       <c r="F6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B8" t="s">
         <v>4</v>
@@ -1375,12 +1381,12 @@
         <v>7</v>
       </c>
       <c r="F8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -1395,12 +1401,12 @@
         <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B10">
         <v>2000</v>
@@ -1412,22 +1418,239 @@
         <v>9</v>
       </c>
       <c r="E10">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="F10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{D0F0CCAB-29C2-4625-A7CC-45A06D76BBB1}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{AD1AC062-4176-4D54-B442-B2EEFF2FDCCD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A2279D5-24C4-4BCD-AFBA-787F1955955C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8D62319-E21E-4172-8A7A-3A90FA780EA4}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="3" width="15.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4">
+        <v>90000</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:B4" xr:uid="{E8D62319-E21E-4172-8A7A-3A90FA780EA4}"/>
+  <hyperlinks>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{9D350AF9-BFE6-4F52-90CD-59B614EC021A}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48B88895-7B00-479C-AEE7-C64182C09A6A}">
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="5" width="15.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:E5" xr:uid="{48B88895-7B00-479C-AEE7-C64182C09A6A}"/>
+  <hyperlinks>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{4ECA5CF2-2425-4D51-A59E-8EC1B379EAA9}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53A36FB9-0062-48CE-BEFC-7770D479615F}">
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="5" width="15.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:E5" xr:uid="{53A36FB9-0062-48CE-BEFC-7770D479615F}"/>
+  <hyperlinks>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{8DF543DD-9ECF-4847-A167-B5D4E29B9B26}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4966192A-9B57-48ED-82CA-07B1F7E843B0}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1441,13 +1664,13 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -1463,7 +1686,7 @@
         <v>8</v>
       </c>
       <c r="B4">
-        <v>90000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
@@ -1471,20 +1694,20 @@
         <v>10</v>
       </c>
       <c r="B5">
-        <v>35000</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:B5" xr:uid="{4A2279D5-24C4-4BCD-AFBA-787F1955955C}"/>
+  <autoFilter ref="A3:B5" xr:uid="{4966192A-9B57-48ED-82CA-07B1F7E843B0}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{4E11CE55-27B5-4461-9D89-7D133EC0D5B6}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{83B5447F-93EB-4ED8-AD6B-45013A8D705D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BE7D445-B4B3-4246-8A8F-FD25D03C9CFF}">
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A5BED0E-0859-44DF-BF46-F7248325736F}">
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1498,13 +1721,13 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -1528,47 +1751,47 @@
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B4">
-        <v>0</v>
+      <c r="B4" t="s">
+        <v>27</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4">
         <v>1</v>
       </c>
       <c r="E4">
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B5">
-        <v>0</v>
+      <c r="B5" t="s">
+        <v>27</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D5">
         <v>1</v>
       </c>
       <c r="E5">
-        <v>35000</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:E5" xr:uid="{7BE7D445-B4B3-4246-8A8F-FD25D03C9CFF}"/>
+  <autoFilter ref="A3:E5" xr:uid="{3A5BED0E-0859-44DF-BF46-F7248325736F}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{A9B0FF47-23BF-4DC5-9E2B-BC405C8B7083}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{1CF7182D-4E08-4605-9609-A22839AC80F4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBEEF758-C502-4933-A2A6-8B1322C8B826}">
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D7EE2E1-1930-46A0-92F2-3CD53E02BD82}">
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1582,13 +1805,13 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>23</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -1612,47 +1835,47 @@
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B4">
-        <v>0</v>
+      <c r="B4" t="s">
+        <v>27</v>
       </c>
       <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4" t="s">
-        <v>9</v>
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>-30</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B5">
-        <v>0</v>
+      <c r="B5" t="s">
+        <v>27</v>
       </c>
       <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5" t="s">
-        <v>9</v>
+        <v>-10000</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:E5" xr:uid="{FBEEF758-C502-4933-A2A6-8B1322C8B826}"/>
+  <autoFilter ref="A3:E5" xr:uid="{2D7EE2E1-1930-46A0-92F2-3CD53E02BD82}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{BB516364-ADBD-48EA-A155-49EF205EF8B1}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{B1EEB487-3696-4EE3-AA26-ADA560FC052B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{858D3F62-F9A8-4F35-B963-FB00C60864A3}">
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E4DBEB7-E478-4CF6-86BE-2C359E0A2471}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1666,13 +1889,13 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -1688,7 +1911,7 @@
         <v>8</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
@@ -1696,238 +1919,13 @@
         <v>10</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>12000</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:B5" xr:uid="{858D3F62-F9A8-4F35-B963-FB00C60864A3}"/>
+  <autoFilter ref="A3:B5" xr:uid="{1E4DBEB7-E478-4CF6-86BE-2C359E0A2471}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{4FB1C5B1-9773-4863-8C8D-FD46E8E20DEF}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21A578FA-B768-4981-B1F5-49AB358DD6FF}">
-  <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="5" width="15.6328125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A3:E5" xr:uid="{21A578FA-B768-4981-B1F5-49AB358DD6FF}"/>
-  <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{BD7BABF1-5C46-4362-A479-9511820438C8}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF7CBC74-6D79-489F-BC3F-767713D66F69}">
-  <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="5" width="15.6328125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5">
-        <v>0</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A3:E5" xr:uid="{CF7CBC74-6D79-489F-BC3F-767713D66F69}"/>
-  <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{13746198-730D-4943-A033-48E53AA0DC56}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{671E0F04-C44D-4A3F-ACBB-69D6B15FEAAF}">
-  <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="3" width="15.6328125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5">
-        <v>12000</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A3:B5" xr:uid="{671E0F04-C44D-4A3F-ACBB-69D6B15FEAAF}"/>
-  <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{01ECC430-2371-4F10-8937-BC7EDB143CD2}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{2BE05E61-47F0-46A4-9378-FF7213FF6890}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>